<commit_message>
move topic and action keyword into GBS Keyword excel file
</commit_message>
<xml_diff>
--- a/GBS Keywords.xlsx
+++ b/GBS Keywords.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/90893d775f8cdf65/Documents/Internship/Degree/AGOS Asia Sdn Bhd/gbs_lead_radar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="11_8D4B8391416375DDD56B79B8F0CC6B0EE64186A1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8754DE2B-D7F4-4498-8319-5342B60A3C3D}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="11_8D4B8391416375DDD56B79B8F0CC6B0EE64186A1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{965FE06A-6991-4420-BB3C-090CB1C28592}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Keywords" sheetId="1" r:id="rId1"/>
+    <sheet name="Topics" sheetId="2" r:id="rId2"/>
+    <sheet name="Actions" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
   <si>
     <t>Keyword</t>
   </si>
@@ -78,6 +80,69 @@
   </si>
   <si>
     <t>"shared services" Penang</t>
+  </si>
+  <si>
+    <t>shared services</t>
+  </si>
+  <si>
+    <t>global capability center</t>
+  </si>
+  <si>
+    <t>centre of excellence</t>
+  </si>
+  <si>
+    <t>set up</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>expand</t>
+  </si>
+  <si>
+    <t>invest</t>
+  </si>
+  <si>
+    <t>Topic</t>
+  </si>
+  <si>
+    <t>global business services</t>
+  </si>
+  <si>
+    <t>global capability centre</t>
+  </si>
+  <si>
+    <t>center of excellence</t>
+  </si>
+  <si>
+    <t>gbs</t>
+  </si>
+  <si>
+    <t>gcc</t>
+  </si>
+  <si>
+    <t>coe</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>setting up</t>
+  </si>
+  <si>
+    <t>establish</t>
+  </si>
+  <si>
+    <t>launch</t>
+  </si>
+  <si>
+    <t>expansion</t>
+  </si>
+  <si>
+    <t>hub</t>
+  </si>
+  <si>
+    <t>announce</t>
   </si>
 </sst>
 </file>
@@ -528,7 +593,144 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03DB85D0-C176-4CD9-8AAF-917A5FD1A09B}">
+  <dimension ref="A1:A10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A8433E5-678A-40C2-A2A6-D3E6533DD1F6}">
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="ef15a170-6792-45de-83de-db50ff6ed40a">
@@ -536,15 +738,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -791,19 +984,19 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F15E30D6-B099-4093-B89D-1EFA692A924E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13E12AA1-198D-4AE4-B691-E044829E62E8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="ef15a170-6792-45de-83de-db50ff6ed40a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F15E30D6-B099-4093-B89D-1EFA692A924E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Added TinyFish for general research and email for report
</commit_message>
<xml_diff>
--- a/GBS Keywords.xlsx
+++ b/GBS Keywords.xlsx
@@ -1,21 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/90893d775f8cdf65/Documents/Internship/Degree/AGOS Asia Sdn Bhd/gbs_lead_radar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="11_8D4B8391416375DDD56B79B8F0CC6B0EE64186A1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{965FE06A-6991-4420-BB3C-090CB1C28592}"/>
+  <xr:revisionPtr revIDLastSave="100" documentId="11_8D4B8391416375DDD56B79B8F0CC6B0EE64186A1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6103AAF-6AAC-4A5B-8C14-B26556E00357}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Keywords" sheetId="1" r:id="rId1"/>
-    <sheet name="Topics" sheetId="2" r:id="rId2"/>
-    <sheet name="Actions" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -41,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="22">
   <si>
     <t>Keyword</t>
   </si>
@@ -64,98 +62,175 @@
     <t>"global capability center" Malaysia</t>
   </si>
   <si>
-    <t>"set up" "shared services centre"</t>
-  </si>
-  <si>
-    <t>"establish" "global business services"</t>
-  </si>
-  <si>
     <t>"regional hub" "shared services" Kuala Lumpur</t>
   </si>
   <si>
-    <t>"centre of excellence" "shared services"</t>
-  </si>
-  <si>
     <t>"GBS" MDEC</t>
   </si>
   <si>
     <t>"shared services" Penang</t>
   </si>
   <si>
-    <t>shared services</t>
-  </si>
-  <si>
-    <t>global capability center</t>
-  </si>
-  <si>
-    <t>centre of excellence</t>
-  </si>
-  <si>
-    <t>set up</t>
-  </si>
-  <si>
-    <t>open</t>
-  </si>
-  <si>
-    <t>expand</t>
-  </si>
-  <si>
-    <t>invest</t>
-  </si>
-  <si>
-    <t>Topic</t>
-  </si>
-  <si>
-    <t>global business services</t>
-  </si>
-  <si>
-    <t>global capability centre</t>
-  </si>
-  <si>
-    <t>center of excellence</t>
-  </si>
-  <si>
-    <t>gbs</t>
-  </si>
-  <si>
-    <t>gcc</t>
-  </si>
-  <si>
-    <t>coe</t>
-  </si>
-  <si>
-    <t>Action</t>
-  </si>
-  <si>
-    <t>setting up</t>
-  </si>
-  <si>
-    <t>establish</t>
-  </si>
-  <si>
-    <t>launch</t>
-  </si>
-  <si>
-    <t>expansion</t>
-  </si>
-  <si>
-    <t>hub</t>
-  </si>
-  <si>
-    <t>announce</t>
+    <r>
+      <t>"new global capability centre"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Malaysia</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>"launches regional hub"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Malaysia</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>"expands global business services"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Malaysia</t>
+    </r>
+  </si>
+  <si>
+    <t>"set up" "shared services centre" Malaysia</t>
+  </si>
+  <si>
+    <t>"establish" "global business services" Malaysia</t>
+  </si>
+  <si>
+    <t>"centre of excellence" "shared services" Malaysia</t>
+  </si>
+  <si>
+    <r>
+      <t>"setting up a shared services centre"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Malaysia</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>"setting up a shared services center"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Malaysia</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>"opening a shared services centre"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Malaysia</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>"opening a shared services center"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Malaysia</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>"building a shared services centre"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Malaysia</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>"building a shared services center"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Malaysia</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -178,8 +253,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -494,13 +570,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="41.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -508,7 +584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -516,7 +592,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -524,7 +600,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -532,7 +608,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -540,180 +616,124 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B6" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="B8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
         <v>8</v>
       </c>
-      <c r="B7" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B9" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="B18" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="B19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B11" t="s">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03DB85D0-C176-4CD9-8AAF-917A5FD1A09B}">
-  <dimension ref="A1:A10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A8433E5-678A-40C2-A2A6-D3E6533DD1F6}">
-  <dimension ref="A1:A11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>33</v>
+      <c r="B20" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -722,25 +742,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ef15a170-6792-45de-83de-db50ff6ed40a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010005D95A1B8F06344DBD080D892BE3A0C3" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee7e3a7599e48882cf636792f97f6c05">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1d9e2a8-36c4-4cdd-a61e-985880338edc" xmlns:ns3="ef15a170-6792-45de-83de-db50ff6ed40a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="323ecb5f9c293f65e7131171c536b2a6" ns2:_="" ns3:_="">
     <xsd:import namespace="d1d9e2a8-36c4-4cdd-a61e-985880338edc"/>
@@ -983,25 +984,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F15E30D6-B099-4093-B89D-1EFA692A924E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ef15a170-6792-45de-83de-db50ff6ed40a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13E12AA1-198D-4AE4-B691-E044829E62E8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ef15a170-6792-45de-83de-db50ff6ed40a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B590D771-F8C1-48FD-A2D7-0589659D0593}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1018,4 +1020,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13E12AA1-198D-4AE4-B691-E044829E62E8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ef15a170-6792-45de-83de-db50ff6ed40a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F15E30D6-B099-4093-B89D-1EFA692A924E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>